<commit_message>
Rezerwa urlopowa: scenariusze testowe (30) i kalkulator zgodne z aktualnymi regulami
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XkLQcV8gkZA892VpAppynM
</commit_message>
<xml_diff>
--- a/Rezerwy urlopowe/Rezerwa Al/Rezerwa urlopowa - scenariusze testowe.xlsx
+++ b/Rezerwy urlopowe/Rezerwa Al/Rezerwa urlopowa - scenariusze testowe.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Kalkulator" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Scenariusze!$A$1:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Scenariusze!$A$1:$I$31</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -56,18 +56,18 @@
     <t>Urlop</t>
   </si>
   <si>
-    <t>Pełny etat, bez zaległego, rezerwa za luty</t>
-  </si>
-  <si>
-    <t>Etat 1/1 od 2020, limit 2026 = 26 dni (208 h), zaległy 0. Urlop wypoczynkowy 3 dni w styczniu (24 h). Pensja 6 000 zł stała, brak zmiennych.</t>
-  </si>
-  <si>
-    <t>1. Kadry i płace → Pracownicy: zaznaczyć pracownika.
-2. Czynności → Nalicz planowane listy płac: definicja „Rezerwa urlopowa”, okres = miesiąc rezerwy, typ wypłaty Etat.
-3. Płace → Planowane listy płac: otworzyć wypłatę pracownika, element „Rezerwa urlopowa” (zakładka Zapis obliczeń).</t>
-  </si>
-  <si>
-    <t>Zaległy 0; bieżący = 208 × 2/12 = 34,67 h = 4,33 dni; wykorzystany 3,00 dni; godziny rezerwy 10,67 h. Podstawa 1 = 6 000,00. Kwota = 10,67 h × 6 000 / (współczynnik × 1) / 8 (patrz arkusz Kalkulator, wiersz RU-01).</t>
+    <t>Kolejny urlop – bieżący proporcjonalny zaokrąglany w górę</t>
+  </si>
+  <si>
+    <t>Etat 1/1, limit 2026 = 26 dni (208 h), znacznik limitu „Pierwszy urlop” = Nie, zaległy 0. Urlop 3 dni (24 h) w styczniu. Pensja 6 000 zł, listy XII–II zatwierdzone. Rezerwa za luty.</t>
+  </si>
+  <si>
+    <t>1. Zatwierdzić listy płac etatowych za miesiąc rezerwy i 2 poprzednie.
+2. Kadry i płace → Pracownicy: zaznaczyć pracownika → Czynności → Nalicz planowane listy płac: definicja „Rezerwa urlopowa”, okres = miesiąc rezerwy, typ wypłaty Etat.
+3. Płace → Planowane listy płac: wypłata pracownika → element „Rezerwa urlopowa” → Zapis obliczeń.</t>
+  </si>
+  <si>
+    <t>[1] Kolejny urlop: 34,67 h = 4,33 dni → zaokrąglone w górę 5 dni = 40,00 h; wykorzystany 3,00 dni; do rezerwy 16,00 h (2,00 dni). Kwota – arkusz Kalkulator, wiersz RU-01.</t>
   </si>
   <si>
     <t>RU-02</t>
@@ -76,10 +76,10 @@
     <t>Zaległy z poprzedniego roku</t>
   </si>
   <si>
-    <t>Jak RU-01, ale zaległy z 2025 = 5 dni (40 h); urlop 10 dni (80 h) do 31.05; rezerwa za maj.</t>
-  </si>
-  <si>
-    <t>Zaległy 5,00 dni; bieżący = 208 × 5/12 = 86,67 h = 10,83 dni; wykorzystany 10,00 dni; rezerwa 46,67 h (5,83 dni).</t>
+    <t>Jak RU-01, zaległy z 2025 = 5 dni (40 h); urlop 10 dni (80 h) do 31.05; rezerwa za maj.</t>
+  </si>
+  <si>
+    <t>Zaległy 5,00 dni; bieżący 208 × 5/12 = 10,83 dni → 11 dni (88 h); wykorzystany 10,00 dni; do rezerwy 48,00 h (6,00 dni).</t>
   </si>
   <si>
     <t>RU-03</t>
@@ -88,49 +88,61 @@
     <t>1/2 etatu</t>
   </si>
   <si>
-    <t>Etat 1/2, limit 26 dni = 104 h, zaległy 0, wykorzystane 16 h do 30.06, pensja 3 000 zł; rezerwa za czerwiec.</t>
-  </si>
-  <si>
-    <t>Bieżący = 104 × 6/12 = 52 h; rezerwa 36 h. Dni w kolumnach liczone po 4 h (8 h × 1/2): bieżący 13,00, wykorzystany 4,00. Stawka 1 h = 3 000 / (współczynnik × 0,5) / 8.</t>
+    <t>Etat 1/2, limit 26 dni = 104 h, kolejny urlop, wykorzystane 16 h do 30.06, pensja 3 000 zł; rezerwa za czerwiec.</t>
+  </si>
+  <si>
+    <t>Dzień urlopu = 4 h (8 h × 1/2). Bieżący 104 × 6/12 = 52 h = 13,00 dni (bez zmiany po zaokrągleniu); wykorzystany 4,00 dni; rezerwa 36 h. Stawka 1 h = 3 000 / (współczynnik × 0,5) / 8.</t>
   </si>
   <si>
     <t>RU-04</t>
   </si>
   <si>
-    <t>Urlop pobrany ponad stan (ujemna rezerwa)</t>
-  </si>
-  <si>
-    <t>Zaległy 0, limit 208 h, w lutym pracownik wykorzystał już 10 dni (80 h).</t>
-  </si>
-  <si>
-    <t>Stan ujemny → rezerwa 0, element nie powstaje (Generuj zerowy = Nie). W Zapisie obliczeń: „Ujemny stan urlopu - rezerwa = 0.”</t>
+    <t>Pierwszy urlop – bez zaokrąglenia</t>
+  </si>
+  <si>
+    <t>Pracownik w pierwszej pracy, limity z znacznikiem „Pierwszy urlop” = Tak (narastająco 1/12).</t>
+  </si>
+  <si>
+    <t>W [1] limity opisane „(pierwszy urlop)”, brak linii „Kolejny urlop: … zaokrąglone w górę”; bieżący = suma proporcjonalna bez zaokrąglenia.</t>
   </si>
   <si>
     <t>RU-05</t>
   </si>
   <si>
+    <t>Urlop pobrany ponad stan</t>
+  </si>
+  <si>
+    <t>Zaległy 0, limit 208 h, do końca lutego wykorzystane 10 dni (80 h).</t>
+  </si>
+  <si>
+    <t>Stan ujemny → „Ujemny stan urlopu - rezerwa = 0.”, element nie powstaje (Generuj zerowy = Nie).</t>
+  </si>
+  <si>
+    <t>RU-06</t>
+  </si>
+  <si>
     <t>Pracownik zwolniony w miesiącu rezerwy</t>
   </si>
   <si>
-    <t>Umowa rozwiązana 15.02.2026 (ekwiwalent na liście głównej). Rezerwa za luty.</t>
-  </si>
-  <si>
-    <t>Pracownik pominięty – brak elementu „Rezerwa urlopowa”.</t>
-  </si>
-  <si>
-    <t>RU-06</t>
+    <t>Umowa rozwiązana 15.02.2026.</t>
+  </si>
+  <si>
+    <t>„Pracownik niezatrudniony na 28.02.2026 - pominięty.” – brak elementu.</t>
+  </si>
+  <si>
+    <t>RU-07</t>
   </si>
   <si>
     <t>Urlop dodatkowy (niepełnosprawność)</t>
   </si>
   <si>
-    <t>Pracownik z limitem urlopu dodatkowego 10 dni oprócz wypoczynkowego.</t>
-  </si>
-  <si>
-    <t>Zaległy/bieżący/wykorzystany obejmują oba limity (wypoczynkowy + dodatkowy) – dwa wpisy „Limit …” w Zapisie obliczeń.</t>
-  </si>
-  <si>
-    <t>RU-07</t>
+    <t>Limit urlopu dodatkowego 10 dni oprócz wypoczynkowego.</t>
+  </si>
+  <si>
+    <t>W [1] osobne linie „Limit …” dla obu limitów; zaokrąglenie w górę osobno dla każdego rodzaju limitu; suma w „Do rezerwy”.</t>
+  </si>
+  <si>
+    <t>RU-08</t>
   </si>
   <si>
     <t>Podstawa 1</t>
@@ -139,85 +151,145 @@
     <t>Składniki zmienne – średnia z 3 miesięcy</t>
   </si>
   <si>
-    <t>Pensja 6 000 w 12/2025, 01/2026, 02/2026. Premia (element wliczany do ekwiwalentu) 1 200 za 12/2025 i 600 za 02/2026. Rezerwa za luty.</t>
-  </si>
-  <si>
-    <t>Podstawa 1 = (6 000 × 3 + 1 800) / 3 = 6 600,00. Składniki liczone wg okresu „za”, nie daty wypłaty.</t>
-  </si>
-  <si>
-    <t>RU-08</t>
+    <t>Pensja 6 000; listy XII/2025, I i II/2026 zatwierdzone. Premia (wliczana do ekwiwalentu) 1 200 za XII i 600 za II. Rezerwa za luty.</t>
+  </si>
+  <si>
+    <t>[3] 3 miesiące z wypłatą; podstawa 1 = (7 200 + 6 000 + 6 600) / 3 = 6 600,00. Składniki wg okresu „za”, nie daty wypłaty.</t>
+  </si>
+  <si>
+    <t>RU-09</t>
   </si>
   <si>
     <t>Podwyżka w trakcie 3 miesięcy</t>
   </si>
   <si>
-    <t>Pensja 6 000 do 31.01.2026, od 01.02.2026 7 000. Rezerwa za luty.</t>
+    <t>Pensja 6 000 do 31.01.2026, od 01.02.2026 7 000; listy XII–II zatwierdzone.</t>
   </si>
   <si>
     <t>Podstawa 1 = (6 000 + 6 000 + 7 000) / 3 = 6 333,33 (zasadnicze nominalne z kartoteki).</t>
   </si>
   <si>
-    <t>RU-09</t>
+    <t>RU-10</t>
+  </si>
+  <si>
+    <t>Miesiąc bez wypłaty pomijany</t>
+  </si>
+  <si>
+    <t>Pensja 6 300; brak listy płac za IX/2026; listy VIII i X zatwierdzone, premia 100 w X. Rezerwa za październik.</t>
+  </si>
+  <si>
+    <t>[3] „2026/09 brak wypłaty - pominięty”; podstawa 1 = (6 300 + 6 400) / 2 = 6 350,00.</t>
+  </si>
+  <si>
+    <t>RU-11</t>
   </si>
   <si>
     <t>Zatrudniony w trakcie okresu</t>
   </si>
   <si>
-    <t>Zatrudnienie od 01.01.2026, pensja 6 000. Rezerwa za luty.</t>
-  </si>
-  <si>
-    <t>Średnia z 2 miesięcy (01 i 02/2026) = 6 000,00 – grudzień pominięty (brak zatrudnienia).</t>
-  </si>
-  <si>
-    <t>RU-10</t>
-  </si>
-  <si>
-    <t>Nieobecność chorobowa nie obniża podstawy</t>
+    <t>Zatrudnienie od 01.01.2026, pensja 6 000; listy I i II zatwierdzone. Rezerwa za luty.</t>
+  </si>
+  <si>
+    <t>[3] „2025/12 brak zatrudnienia - pominięty”; średnia z 2 miesięcy = 6 000,00.</t>
+  </si>
+  <si>
+    <t>RU-12</t>
+  </si>
+  <si>
+    <t>Niepełny miesiąc zatrudnienia – wartości nominalne</t>
+  </si>
+  <si>
+    <t>Zatrudnienie od 15.09.2026, pensja 6 000, premia z kartoteki 300 (naliczona proporcjonalnie), nadgodziny 200 za IX (wliczane do ekwiwalentu); X: 6 000 + 300. Rezerwa za październik.</t>
+  </si>
+  <si>
+    <t>[3] 2026/09 z dopiskiem „niepełne zatrudnienie … przelicznik normy (norma IX / norma 15–30.IX)”: zasadnicze 6 000, premia 300 (z kartoteki), nadgodziny 200 × przelicznik. Średnia z IX i X.</t>
+  </si>
+  <si>
+    <t>RU-13</t>
+  </si>
+  <si>
+    <t>Chorobowe nie obniża podstawy</t>
   </si>
   <si>
     <t>Pensja 6 000; w styczniu 10 dni chorobowego (zasadnicze naliczone pomniejszone).</t>
   </si>
   <si>
-    <t>Podstawa 1 = 6 000,00 (zasadnicze nominalne). Przy przełączniku ZASADNICZE_NOMINALNE = false podstawa byłaby niższa – decyzja klienta.</t>
-  </si>
-  <si>
-    <t>RU-11</t>
+    <t>Podstawa 1 = 6 000,00 (zasadnicze nominalne). Przy ZASADNICZE_NOMINALNE = false podstawa byłaby niższa.</t>
+  </si>
+  <si>
+    <t>RU-14</t>
+  </si>
+  <si>
+    <t>Podstawa 1/2</t>
+  </si>
+  <si>
+    <t>Niezatwierdzona lista płac w miesiącu rezerwy</t>
+  </si>
+  <si>
+    <t>Lista płac za X/2026 naliczona, NIEzatwierdzona; przy naliczaniu planu parametr „Uwzględniaj niezatwierdzone listy płac” = Nie.</t>
+  </si>
+  <si>
+    <t>Na górze „UWAGA: brak wypłaty za 2026/10 …”; [3] „2026/10 brak wypłaty - pominięty”; [4] „standard naliczył elementy miesiąca na nowo”. Powtórzyć z parametrem = Tak → brak UWAGA, obie podstawy z listy X.</t>
+  </si>
+  <si>
+    <t>RU-15</t>
   </si>
   <si>
     <t>Podstawa 2</t>
   </si>
   <si>
-    <t>Zgodność ze standardowym ekwiwalentem enova</t>
-  </si>
-  <si>
-    <t>Dowolny pracownik z RU-01/RU-07.</t>
-  </si>
-  <si>
-    <t>1. Kadry i płace → Pracownicy: zaznaczyć pracownika.
-2. Czynności → Nalicz planowane listy płac: definicja „Rezerwa urlopowa”, okres = miesiąc rezerwy, typ wypłaty Etat.
-3. Płace → Planowane listy płac: otworzyć wypłatę pracownika, element „Rezerwa urlopowa” (zakładka Zapis obliczeń).
-4. Porównać z podglądem podstawy ekwiwalentu (element „Ekwiwalent za czas urlopu”) dla tego samego miesiąca.</t>
-  </si>
-  <si>
-    <t>Podstawa 2 za 1 dzień i za 1 godzinę (Zapis obliczeń, sekcja „NALICZANIE EKWIWALENTU”) równa podstawie standardowego ekwiwalentu.</t>
-  </si>
-  <si>
-    <t>RU-12</t>
+    <t>Zgodność ze standardowym ekwiwalentem</t>
+  </si>
+  <si>
+    <t>Pracownik z RU-08; Zapis obliczeń w definicji = „Rezerwa urlopowa,Urlop”.</t>
+  </si>
+  <si>
+    <t>[4] podstawa za dzień i za godzinę równa logowi „NALICZANIE EKWIWALENTU…” (PODSTAWA ZA 1 DZIEŃ / ZA 1 GODZINĘ) widocznemu pod sekcją.</t>
+  </si>
+  <si>
+    <t>RU-16</t>
+  </si>
+  <si>
+    <t>Wynik</t>
+  </si>
+  <si>
+    <t>Wariant podstawy</t>
+  </si>
+  <si>
+    <t>Pracownik z RU-10. W kodzie algorytmu WARIANT_PODSTAWY = 1, potem 2, potem 3.</t>
+  </si>
+  <si>
+    <t>[5] „wariant 1 (podstawa 1)”, „wariant 2 (podstawa 2)”, „wariant 3 (wyższa z podstaw)” – kwota = godziny × odpowiednia stawka 1 h.</t>
+  </si>
+  <si>
+    <t>RU-17</t>
   </si>
   <si>
     <t>Współczynnik</t>
   </si>
   <si>
-    <t>Współczynnik do ekwiwalentu z konfiguracji</t>
-  </si>
-  <si>
-    <t>Konfiguracja → Płace → Nieobecności: „Średnia wg konfiguracji” = Tak, średnia norma miesięczna na 2026 wpisana.</t>
-  </si>
-  <si>
-    <t>W Zapisie obliczeń „Współczynnik do ekwiwalentu” = wartość z konfiguracji × wymiar etatu. Bez konfiguracji: dni robocze roku / 12.</t>
-  </si>
-  <si>
-    <t>RU-13</t>
+    <t>Współczynnik z konfiguracji</t>
+  </si>
+  <si>
+    <t>Konfiguracja → Płace → Nieobecności → Średnia norma miesięczna na 2026 = 20,92.</t>
+  </si>
+  <si>
+    <t>[2] „WSPÓŁCZYNNIK: 20,92 x wymiar 1/1 = 20,92; 8,00 h w dniu urlopu” – zawsze z konfiguracji (niezależnie od „Średnia wg konfiguracji”).</t>
+  </si>
+  <si>
+    <t>RU-18</t>
+  </si>
+  <si>
+    <t>Brak współczynnika w konfiguracji</t>
+  </si>
+  <si>
+    <t>Średnia norma miesięczna na rok rezerwy = 0 (brak wpisu).</t>
+  </si>
+  <si>
+    <t>[2] „UWAGA: brak współczynnika do ekwiwalentu w konfiguracji … - rezerwa = 0.” – element nie powstaje, sekcje [3]–[5] nie występują.</t>
+  </si>
+  <si>
+    <t>RU-19</t>
   </si>
   <si>
     <t>Narzuty</t>
@@ -229,10 +301,10 @@
     <t>Pracownik z RU-01, standardowe stawki ZUS pracodawcy.</t>
   </si>
   <si>
-    <t>Narzuty elementu = emerytalna 9,76% + rentowa 6,50% + wypadkowa (stopa firmy) + FP 2,45% + FGŚP 0,10% od kwoty rezerwy (z uwzględnieniem zwolnień FP/FGŚP i limitu 30-krotności – tak jak liczy silnik płac).</t>
-  </si>
-  <si>
-    <t>RU-14</t>
+    <t>Narzuty elementu = emerytalna 9,76% + rentowa 6,50% + wypadkowa (stopa firmy) + FP 2,45% + FGŚP 0,10% od kwoty rezerwy (zwolnienia FP/FGŚP i limit 30-krotności wg silnika płac). PPK pracodawcy nie wchodzi.</t>
+  </si>
+  <si>
+    <t>RU-20</t>
   </si>
   <si>
     <t>Bezpieczeństwo</t>
@@ -247,22 +319,31 @@
     <t>1. Naliczyć zwykłą listę płac etatowych za luty.</t>
   </si>
   <si>
-    <t>Brak elementów „Rezerwa urlopowa” i „Budżet rezerwy urlopowej” na wypłacie (Rodzaj naliczania = Tylko planowane, Do wypłaty = Nie).</t>
-  </si>
-  <si>
-    <t>RU-15</t>
-  </si>
-  <si>
-    <t>Planowanie po zamknięciu listy płac</t>
-  </si>
-  <si>
-    <t>Lista płac za luty zatwierdzona.</t>
-  </si>
-  <si>
-    <t>Naliczenie planu nie usuwa wypłat z listy głównej. UWAGA: niezatwierdzone wypłaty etatowe pracownika silnik planu USUWA przed naliczeniem – rezerwę liczyć po zatwierdzeniu list płac miesiąca.</t>
-  </si>
-  <si>
-    <t>RU-16</t>
+    <t>Brak elementów „Rezerwa urlopowa” i „Budżet rezerwy urlopowej” (Rodzaj naliczania = Tylko planowane, Do wypłaty = Nie).</t>
+  </si>
+  <si>
+    <t>RU-21</t>
+  </si>
+  <si>
+    <t>Plan</t>
+  </si>
+  <si>
+    <t>Numeracja planowanych list – kilka wydziałów</t>
+  </si>
+  <si>
+    <t>Pracownicy z dwóch różnych wydziałów, rezerwa za 10/2026.</t>
+  </si>
+  <si>
+    <t>1. Zatwierdzić listy płac etatowych za miesiąc rezerwy i 2 poprzednie.
+2. Kadry i płace → Pracownicy: zaznaczyć pracowników obu wydziałów → Czynności → Nalicz planowane listy płac: definicja „Rezerwa urlopowa”, okres = miesiąc rezerwy, typ wypłaty Etat.
+3. Płace → Planowane listy płac: wypłata pracownika → element „Rezerwa urlopowa” → Zapis obliczeń.
+4. Zapisać.</t>
+  </si>
+  <si>
+    <t>Dwie planowane listy REZURL/2026/10/1 i REZURL/2026/10/2; zapis bez błędu „Istnieje już inny zapis w kluczu Numer.WgNumeruDokumentu”.</t>
+  </si>
+  <si>
+    <t>RU-22</t>
   </si>
   <si>
     <t>Budżet</t>
@@ -271,24 +352,23 @@
     <t>Budżet w sierpniu – symulacja limitu na 01.01.2027</t>
   </si>
   <si>
-    <t>Limit 2026 = 26 dni; wykorzystane w 2026 (łącznie z już wprowadzonymi urlopami na IX–XII) = 18 dni; staż daje 26 dni na 2027. Okres planu 08/2026.</t>
-  </si>
-  <si>
-    <t>1. Kadry i płace → Pracownicy: zaznaczyć pracownika.
-2. Nalicz planowane listy płac: definicja „Budżet rezerwy urlopowej”, okres 08/2026.
-3. Sprawdzić element „Budżet rezerwy urlopowej” i jego Zapis obliczeń.</t>
-  </si>
-  <si>
-    <t>Zaległy na 01.01.2027 = 8,00 dni; limit 2027 = 26,00 dni; godziny budżetu 272 h; podstawy 1 i 2 z 06–08/2026.</t>
-  </si>
-  <si>
-    <t>RU-17</t>
+    <t>Limit 2026 = 26 dni; wykorzystane w 2026 (łącznie z wprowadzonymi urlopami na IX–XII) = 18 dni; staż daje 26 dni na 2027.</t>
+  </si>
+  <si>
+    <t>1. Kadry i płace → Pracownicy: zaznaczyć pracownika → Nalicz planowane listy płac: definicja „Budżet rezerwy urlopowej”, okres 08/2026.
+2. Element „Budżet rezerwy urlopowej” → Zapis obliczeń.</t>
+  </si>
+  <si>
+    <t>[1] „Zaległy na 01.01.2027” 8,00 dni, „Limit na rok 2027” 26,00 dni, do rezerwy 272 h (34 dni); podstawy z VI–VIII/2026.</t>
+  </si>
+  <si>
+    <t>RU-23</t>
   </si>
   <si>
     <t>Symulacja nie zapisuje limitów</t>
   </si>
   <si>
-    <t>Po RU-16.</t>
+    <t>Po RU-22.</t>
   </si>
   <si>
     <t>1. Kartoteka pracownika → Limity nieobecności.</t>
@@ -297,7 +377,7 @@
     <t>Brak limitu na rok 2027 (symulacja w niezapisywanej sesji).</t>
   </si>
   <si>
-    <t>RU-18</t>
+    <t>RU-24</t>
   </si>
   <si>
     <t>Zmiana wymiaru urlopu z 20 na 26 dni w 2027</t>
@@ -306,29 +386,56 @@
     <t>Pracownik osiąga 10 lat stażu urlopowego w 03/2027.</t>
   </si>
   <si>
-    <t>Limit 2027 z symulacji = wartość, jaką da „Limity nieobecności / Nalicz” na 2027 (proporcja 20/26 wg zasad enova).</t>
-  </si>
-  <si>
-    <t>RU-19</t>
+    <t>Limit 2027 z symulacji = wartość, jaką da „Limity nieobecności / Nalicz” na 2027.</t>
+  </si>
+  <si>
+    <t>RU-25</t>
+  </si>
+  <si>
+    <t>Zapis obliczeń</t>
+  </si>
+  <si>
+    <t>Uporządkowany log</t>
+  </si>
+  <si>
+    <t>Zapis obliczeń w definicji = „Rezerwa urlopowa”.</t>
+  </si>
+  <si>
+    <t>Nagłówek „=== REZERWA URLOPOWA RRRR/MM - pracownik ===”, sekcje [1] stan urlopu (tabelka godz./dni), [2] współczynnik, [3] podstawa 1, [4] podstawa 2, [5] wynik. Brak obcych logów (np. wyrównania do najniższego).</t>
+  </si>
+  <si>
+    <t>RU-26</t>
+  </si>
+  <si>
+    <t>Log z pełnym standardem</t>
+  </si>
+  <si>
+    <t>Zapis obliczeń w definicji = „Rezerwa urlopowa,Urlop”.</t>
+  </si>
+  <si>
+    <t>Jak RU-25 + pełny log „NALICZANIE EKWIWALENTU ZA URLOP WYPOCZYNKOWY” w sekcji [4].</t>
+  </si>
+  <si>
+    <t>RU-27</t>
   </si>
   <si>
     <t>Widok</t>
   </si>
   <si>
-    <t>Widok rezerwy na liście Pracownicy</t>
+    <t>Kolumny widoku rezerwy</t>
   </si>
   <si>
     <t>Plan „Rezerwa urlopowa” za 02/2026 naliczony.</t>
   </si>
   <si>
-    <t>1. Pracownicy, Aktualność = 28.02.2026.
-2. Ustawienia kolumn → kategoria „Rezerwa urlopowa”: Kod, Imię, Nazwisko, Rezerwa MPK, … Rezerwa narzuty.</t>
-  </si>
-  <si>
-    <t>Kolumny pokazują wartości z elementu planu za luty. Aktualność 31.03 (brak planu) → zera.</t>
-  </si>
-  <si>
-    <t>RU-20</t>
+    <t>1. Kadry i płace → Pracownicy, Aktualność = ostatni dzień miesiąca rezerwy.
+2. Ustawienia kolumn → kategoria „Rezerwa urlopowa”: Kod, Imię, Nazwisko, Rezerwa MPK … Rezerwa narzuty.</t>
+  </si>
+  <si>
+    <t>Kolumny = wartości elementu planu za luty (zaległy/bieżący/wykorzystany w dniach, godziny, podstawy 1 i 2, kwota, narzuty). Aktualność 31.03 (brak planu) → zera.</t>
+  </si>
+  <si>
+    <t>RU-28</t>
   </si>
   <si>
     <t>Ponowne naliczenie planu</t>
@@ -337,13 +444,10 @@
     <t>Plan za 02/2026 naliczony dwa razy (np. po korekcie urlopu).</t>
   </si>
   <si>
-    <t>Jak RU-19.</t>
-  </si>
-  <si>
     <t>Kolumny pokazują wynik ostatniego naliczenia.</t>
   </si>
   <si>
-    <t>RU-21</t>
+    <t>RU-29</t>
   </si>
   <si>
     <t>MPK z wydziału nadrzędnego</t>
@@ -355,10 +459,26 @@
     <t>Rezerwa MPK = X.</t>
   </si>
   <si>
+    <t>RU-30</t>
+  </si>
+  <si>
+    <t>Kolumny budżetu</t>
+  </si>
+  <si>
+    <t>Plan „Budżet rezerwy urlopowej” za 08/2026 naliczony.</t>
+  </si>
+  <si>
+    <t>1. Kadry i płace → Pracownicy, Aktualność = dowolny dzień sierpnia 2026.
+2. Ustawienia kolumn → kategoria „Rezerwa urlopowa”: Kod, Imię, Nazwisko, Rezerwa MPK, Budżet ….</t>
+  </si>
+  <si>
+    <t>Kolumny „Budżet …” = wartości elementu budżetu z RU-22; kolumny „Rezerwa …” niezależne (inny element).</t>
+  </si>
+  <si>
     <t>Wymiar etatu</t>
   </si>
   <si>
-    <t>Godzin w dniu urlopu (8)</t>
+    <t>Godzin w dniu (8)</t>
   </si>
   <si>
     <t>Współczynnik do ekwiwalentu</t>
@@ -373,22 +493,19 @@
     <t>Miesiąc rezerwy (1-12)</t>
   </si>
   <si>
+    <t>Pierwszy urlop (1/0)</t>
+  </si>
+  <si>
     <t>Wykorzystany (h)</t>
   </si>
   <si>
-    <t>Zasadnicze M-2</t>
-  </si>
-  <si>
-    <t>Zasadnicze M-1</t>
-  </si>
-  <si>
-    <t>Zasadnicze M</t>
-  </si>
-  <si>
-    <t>Zmienne razem 3 mies.</t>
-  </si>
-  <si>
-    <t>Liczba miesięcy zatrudnienia (1-3)</t>
+    <t>M-2 razem (puste = brak wypłaty)</t>
+  </si>
+  <si>
+    <t>M-1 razem</t>
+  </si>
+  <si>
+    <t>M razem</t>
   </si>
   <si>
     <t>Bieżący prop. (h)</t>
@@ -412,7 +529,13 @@
     <t>Wykorzystany (dni)</t>
   </si>
   <si>
-    <t>Współczynnik 20,83 to przykład – wpisać wartość z konfiguracji enova (średnia norma miesięczna na dany rok). Zielone kolumny liczą się formułami, tak samo jak algorytm elementu (wariant podstawy 1).</t>
+    <t>Kolumny M-2 / M-1 / M = zasadnicze nominalne + składniki wliczane do ekwiwalentu za miesiąc; PUSTE = brak wypłaty (miesiąc pomijany w średniej, jak w podstawie 2).</t>
+  </si>
+  <si>
+    <t>Współczynnik 20,92 = wartość z konfiguracji bazy (średnia norma miesięczna); 0 = brak rezerwy.</t>
+  </si>
+  <si>
+    <t>Zielone kolumny liczą się formułami tak samo jak algorytm elementu (wariant podstawy 1).</t>
   </si>
 </sst>
 </file>
@@ -795,7 +918,7 @@
     <col min="3" max="3" width="30.710938" customWidth="1"/>
     <col min="4" max="4" width="48.710938" customWidth="1"/>
     <col min="5" max="5" width="42.710938" customWidth="1"/>
-    <col min="6" max="6" width="55.710938" customWidth="1"/>
+    <col min="6" max="6" width="60.710938" customWidth="1"/>
     <col min="7" max="7" width="30.710938" customWidth="1"/>
     <col min="8" max="8" width="12.7109375" customWidth="1"/>
     <col min="9" max="9" width="30.710938" customWidth="1"/>
@@ -830,7 +953,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="120">
+    <row r="2" ht="135">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -853,7 +976,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
-    <row r="3" ht="120">
+    <row r="3" ht="135">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -876,7 +999,7 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" ht="120">
+    <row r="4" ht="135">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -899,7 +1022,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" ht="120">
+    <row r="5" ht="135">
       <c r="A5" s="2" t="s">
         <v>23</v>
       </c>
@@ -922,7 +1045,7 @@
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" ht="120">
+    <row r="6" ht="135">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -945,7 +1068,7 @@
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" ht="120">
+    <row r="7" ht="135">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -968,35 +1091,35 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" ht="120">
+    <row r="8" ht="135">
       <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
     </row>
-    <row r="9" ht="120">
+    <row r="9" ht="135">
       <c r="A9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>41</v>
@@ -1014,12 +1137,12 @@
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
     </row>
-    <row r="10" ht="120">
+    <row r="10" ht="135">
       <c r="A10" s="2" t="s">
         <v>44</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>45</v>
@@ -1037,12 +1160,12 @@
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" ht="120">
+    <row r="11" ht="135">
       <c r="A11" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>49</v>
@@ -1060,208 +1183,208 @@
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
     </row>
-    <row r="12" ht="165">
+    <row r="12" ht="135">
       <c r="A12" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
     </row>
-    <row r="13" ht="120">
+    <row r="13" ht="135">
       <c r="A13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
     </row>
-    <row r="14" ht="120">
+    <row r="14" ht="135">
       <c r="A14" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
     </row>
-    <row r="15" ht="45">
+    <row r="15" ht="135">
       <c r="A15" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
     </row>
-    <row r="16" ht="120">
+    <row r="16" ht="135">
       <c r="A16" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
     </row>
-    <row r="17" ht="90">
+    <row r="17" ht="135">
       <c r="A17" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>83</v>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
     </row>
-    <row r="18" ht="30">
+    <row r="18" ht="135">
       <c r="A18" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>87</v>
+        <v>13</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
     </row>
-    <row r="19" ht="90">
+    <row r="19" ht="135">
       <c r="A19" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>82</v>
+        <v>13</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
     </row>
-    <row r="20" ht="60">
+    <row r="20" ht="135">
       <c r="A20" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>97</v>
+        <v>13</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
@@ -1269,52 +1392,259 @@
     </row>
     <row r="21" ht="30">
       <c r="A21" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>94</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
     </row>
-    <row r="22" ht="30">
+    <row r="22" ht="165">
       <c r="A22" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
     </row>
+    <row r="23" ht="90">
+      <c r="A23" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+    </row>
+    <row r="24" ht="30">
+      <c r="A24" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+    </row>
+    <row r="25" ht="90">
+      <c r="A25" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+    </row>
+    <row r="26" ht="135">
+      <c r="A26" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+    </row>
+    <row r="27" ht="135">
+      <c r="A27" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+    </row>
+    <row r="28" ht="75">
+      <c r="A28" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+    </row>
+    <row r="29" ht="75">
+      <c r="A29" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+    </row>
+    <row r="30" ht="75">
+      <c r="A30" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+    </row>
+    <row r="31" ht="75">
+      <c r="A31" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I22"/>
+  <autoFilter ref="A1:I31"/>
 </worksheet>
 </file>
 
@@ -1342,72 +1672,68 @@
     <col min="18" max="18" width="13.7109375" customWidth="1"/>
     <col min="19" max="19" width="13.7109375" customWidth="1"/>
     <col min="20" max="20" width="13.7109375" customWidth="1"/>
-    <col min="21" max="21" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="60">
+    <row r="1" ht="45">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>108</v>
+        <v>148</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>109</v>
+        <v>149</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>111</v>
+        <v>151</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>112</v>
+        <v>152</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>113</v>
+        <v>153</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>114</v>
+        <v>154</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>115</v>
+        <v>155</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>116</v>
+        <v>156</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>117</v>
+        <v>157</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>119</v>
+        <v>158</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>159</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>121</v>
+        <v>40</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>36</v>
+        <v>161</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>122</v>
+        <v>162</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>123</v>
+        <v>163</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>124</v>
+        <v>164</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>126</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2">
@@ -1421,7 +1747,7 @@
         <v>8</v>
       </c>
       <c r="D2">
-        <v>20.829999999999998</v>
+        <v>20.920000000000002</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1433,10 +1759,10 @@
         <v>2</v>
       </c>
       <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
         <v>24</v>
-      </c>
-      <c r="I2">
-        <v>6000</v>
       </c>
       <c r="J2">
         <v>6000</v>
@@ -1445,41 +1771,38 @@
         <v>6000</v>
       </c>
       <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>3</v>
+        <v>6000</v>
+      </c>
+      <c r="M2" s="5">
+        <f>IF(H2=1,F2*G2/12,CEILING(ROUND(F2*G2/12/(C2*B2),6),1)*C2*B2)</f>
+        <v>40</v>
       </c>
       <c r="N2" s="5">
-        <f>F2*G2/12</f>
-        <v>34.666666666666664</v>
+        <f>MAX(0,E2+M2-I2)</f>
+        <v>16</v>
       </c>
       <c r="O2" s="5">
-        <f>MAX(0,E2+N2-H2)</f>
-        <v>10.666666666666664</v>
-      </c>
-      <c r="P2" s="5">
-        <f>ROUND((I2+J2+K2+L2)/M2,2)</f>
+        <f>ROUND(AVERAGE(J2:L2),2)</f>
         <v>6000</v>
       </c>
-      <c r="Q2" s="6">
-        <f>P2/(D2*B2)/C2</f>
-        <v>36.005760921747481</v>
+      <c r="P2" s="6">
+        <f>O2/(D2*B2)/C2</f>
+        <v>35.850860420650093</v>
+      </c>
+      <c r="Q2" s="5">
+        <f>ROUND(N2*P2,2)</f>
+        <v>573.61000000000001</v>
       </c>
       <c r="R2" s="5">
-        <f>ROUND(O2*Q2,2)</f>
-        <v>384.06</v>
+        <f>ROUND(E2/(C2*B2),2)</f>
+        <v>0</v>
       </c>
       <c r="S2" s="5">
-        <f>ROUND(E2/(C2*B2),2)</f>
-        <v>0</v>
+        <f>ROUND(M2/(C2*B2),2)</f>
+        <v>5</v>
       </c>
       <c r="T2" s="5">
-        <f>ROUND(N2/(C2*B2),2)</f>
-        <v>4.3300000000000001</v>
-      </c>
-      <c r="U2" s="5">
-        <f>ROUND(H2/(C2*B2),2)</f>
+        <f>ROUND(I2/(C2*B2),2)</f>
         <v>3</v>
       </c>
     </row>
@@ -1494,7 +1817,7 @@
         <v>8</v>
       </c>
       <c r="D3">
-        <v>20.829999999999998</v>
+        <v>20.920000000000002</v>
       </c>
       <c r="E3">
         <v>40</v>
@@ -1506,10 +1829,10 @@
         <v>5</v>
       </c>
       <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
         <v>80</v>
-      </c>
-      <c r="I3">
-        <v>6000</v>
       </c>
       <c r="J3">
         <v>6000</v>
@@ -1518,41 +1841,38 @@
         <v>6000</v>
       </c>
       <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>3</v>
+        <v>6000</v>
+      </c>
+      <c r="M3" s="5">
+        <f>IF(H3=1,F3*G3/12,CEILING(ROUND(F3*G3/12/(C3*B3),6),1)*C3*B3)</f>
+        <v>88</v>
       </c>
       <c r="N3" s="5">
-        <f>F3*G3/12</f>
-        <v>86.666666666666671</v>
+        <f>MAX(0,E3+M3-I3)</f>
+        <v>48</v>
       </c>
       <c r="O3" s="5">
-        <f>MAX(0,E3+N3-H3)</f>
-        <v>46.666666666666671</v>
-      </c>
-      <c r="P3" s="5">
-        <f>ROUND((I3+J3+K3+L3)/M3,2)</f>
+        <f>ROUND(AVERAGE(J3:L3),2)</f>
         <v>6000</v>
       </c>
-      <c r="Q3" s="6">
-        <f>P3/(D3*B3)/C3</f>
-        <v>36.005760921747481</v>
+      <c r="P3" s="6">
+        <f>O3/(D3*B3)/C3</f>
+        <v>35.850860420650093</v>
+      </c>
+      <c r="Q3" s="5">
+        <f>ROUND(N3*P3,2)</f>
+        <v>1720.8399999999999</v>
       </c>
       <c r="R3" s="5">
-        <f>ROUND(O3*Q3,2)</f>
-        <v>1680.27</v>
-      </c>
-      <c r="S3" s="5">
         <f>ROUND(E3/(C3*B3),2)</f>
         <v>5</v>
       </c>
+      <c r="S3" s="5">
+        <f>ROUND(M3/(C3*B3),2)</f>
+        <v>11</v>
+      </c>
       <c r="T3" s="5">
-        <f>ROUND(N3/(C3*B3),2)</f>
-        <v>10.83</v>
-      </c>
-      <c r="U3" s="5">
-        <f>ROUND(H3/(C3*B3),2)</f>
+        <f>ROUND(I3/(C3*B3),2)</f>
         <v>10</v>
       </c>
     </row>
@@ -1567,7 +1887,7 @@
         <v>8</v>
       </c>
       <c r="D4">
-        <v>20.829999999999998</v>
+        <v>20.920000000000002</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1579,10 +1899,10 @@
         <v>6</v>
       </c>
       <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
         <v>16</v>
-      </c>
-      <c r="I4">
-        <v>3000</v>
       </c>
       <c r="J4">
         <v>3000</v>
@@ -1591,47 +1911,44 @@
         <v>3000</v>
       </c>
       <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>3</v>
+        <v>3000</v>
+      </c>
+      <c r="M4" s="5">
+        <f>IF(H4=1,F4*G4/12,CEILING(ROUND(F4*G4/12/(C4*B4),6),1)*C4*B4)</f>
+        <v>52</v>
       </c>
       <c r="N4" s="5">
-        <f>F4*G4/12</f>
-        <v>52</v>
+        <f>MAX(0,E4+M4-I4)</f>
+        <v>36</v>
       </c>
       <c r="O4" s="5">
-        <f>MAX(0,E4+N4-H4)</f>
-        <v>36</v>
-      </c>
-      <c r="P4" s="5">
-        <f>ROUND((I4+J4+K4+L4)/M4,2)</f>
+        <f>ROUND(AVERAGE(J4:L4),2)</f>
         <v>3000</v>
       </c>
-      <c r="Q4" s="6">
-        <f>P4/(D4*B4)/C4</f>
-        <v>36.005760921747481</v>
+      <c r="P4" s="6">
+        <f>O4/(D4*B4)/C4</f>
+        <v>35.850860420650093</v>
+      </c>
+      <c r="Q4" s="5">
+        <f>ROUND(N4*P4,2)</f>
+        <v>1290.6300000000001</v>
       </c>
       <c r="R4" s="5">
-        <f>ROUND(O4*Q4,2)</f>
-        <v>1296.21</v>
+        <f>ROUND(E4/(C4*B4),2)</f>
+        <v>0</v>
       </c>
       <c r="S4" s="5">
-        <f>ROUND(E4/(C4*B4),2)</f>
-        <v>0</v>
+        <f>ROUND(M4/(C4*B4),2)</f>
+        <v>13</v>
       </c>
       <c r="T4" s="5">
-        <f>ROUND(N4/(C4*B4),2)</f>
-        <v>13</v>
-      </c>
-      <c r="U4" s="5">
-        <f>ROUND(H4/(C4*B4),2)</f>
+        <f>ROUND(I4/(C4*B4),2)</f>
         <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -1640,7 +1957,7 @@
         <v>8</v>
       </c>
       <c r="D5">
-        <v>20.829999999999998</v>
+        <v>20.920000000000002</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1649,13 +1966,13 @@
         <v>208</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H5">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="J5">
         <v>6000</v>
@@ -1664,47 +1981,44 @@
         <v>6000</v>
       </c>
       <c r="L5">
-        <v>1800</v>
-      </c>
-      <c r="M5">
-        <v>3</v>
+        <v>6000</v>
+      </c>
+      <c r="M5" s="5">
+        <f>IF(H5=1,F5*G5/12,CEILING(ROUND(F5*G5/12/(C5*B5),6),1)*C5*B5)</f>
+        <v>173.33333333333334</v>
       </c>
       <c r="N5" s="5">
-        <f>F5*G5/12</f>
-        <v>34.666666666666664</v>
+        <f>MAX(0,E5+M5-I5)</f>
+        <v>173.33333333333334</v>
       </c>
       <c r="O5" s="5">
-        <f>MAX(0,E5+N5-H5)</f>
-        <v>10.666666666666664</v>
-      </c>
-      <c r="P5" s="5">
-        <f>ROUND((I5+J5+K5+L5)/M5,2)</f>
-        <v>6600</v>
-      </c>
-      <c r="Q5" s="6">
-        <f>P5/(D5*B5)/C5</f>
-        <v>39.606337013922229</v>
+        <f>ROUND(AVERAGE(J5:L5),2)</f>
+        <v>6000</v>
+      </c>
+      <c r="P5" s="6">
+        <f>O5/(D5*B5)/C5</f>
+        <v>35.850860420650093</v>
+      </c>
+      <c r="Q5" s="5">
+        <f>ROUND(N5*P5,2)</f>
+        <v>6214.1499999999996</v>
       </c>
       <c r="R5" s="5">
-        <f>ROUND(O5*Q5,2)</f>
-        <v>422.47000000000003</v>
+        <f>ROUND(E5/(C5*B5),2)</f>
+        <v>0</v>
       </c>
       <c r="S5" s="5">
-        <f>ROUND(E5/(C5*B5),2)</f>
-        <v>0</v>
+        <f>ROUND(M5/(C5*B5),2)</f>
+        <v>21.670000000000002</v>
       </c>
       <c r="T5" s="5">
-        <f>ROUND(N5/(C5*B5),2)</f>
-        <v>4.3300000000000001</v>
-      </c>
-      <c r="U5" s="5">
-        <f>ROUND(H5/(C5*B5),2)</f>
-        <v>3</v>
+        <f>ROUND(I5/(C5*B5),2)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -1713,7 +2027,7 @@
         <v>8</v>
       </c>
       <c r="D6">
-        <v>20.829999999999998</v>
+        <v>20.920000000000002</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1725,53 +2039,50 @@
         <v>2</v>
       </c>
       <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
         <v>24</v>
       </c>
-      <c r="I6">
+      <c r="J6">
+        <v>7200</v>
+      </c>
+      <c r="K6">
         <v>6000</v>
       </c>
-      <c r="J6">
-        <v>6000</v>
-      </c>
-      <c r="K6">
-        <v>7000</v>
-      </c>
       <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>3</v>
+        <v>6600</v>
+      </c>
+      <c r="M6" s="5">
+        <f>IF(H6=1,F6*G6/12,CEILING(ROUND(F6*G6/12/(C6*B6),6),1)*C6*B6)</f>
+        <v>40</v>
       </c>
       <c r="N6" s="5">
-        <f>F6*G6/12</f>
-        <v>34.666666666666664</v>
+        <f>MAX(0,E6+M6-I6)</f>
+        <v>16</v>
       </c>
       <c r="O6" s="5">
-        <f>MAX(0,E6+N6-H6)</f>
-        <v>10.666666666666664</v>
-      </c>
-      <c r="P6" s="5">
-        <f>ROUND((I6+J6+K6+L6)/M6,2)</f>
-        <v>6333.3299999999999</v>
-      </c>
-      <c r="Q6" s="6">
-        <f>P6/(D6*B6)/C6</f>
-        <v>38.006060969755161</v>
+        <f>ROUND(AVERAGE(J6:L6),2)</f>
+        <v>6600</v>
+      </c>
+      <c r="P6" s="6">
+        <f>O6/(D6*B6)/C6</f>
+        <v>39.435946462715101</v>
+      </c>
+      <c r="Q6" s="5">
+        <f>ROUND(N6*P6,2)</f>
+        <v>630.98000000000002</v>
       </c>
       <c r="R6" s="5">
-        <f>ROUND(O6*Q6,2)</f>
-        <v>405.39999999999998</v>
+        <f>ROUND(E6/(C6*B6),2)</f>
+        <v>0</v>
       </c>
       <c r="S6" s="5">
-        <f>ROUND(E6/(C6*B6),2)</f>
-        <v>0</v>
+        <f>ROUND(M6/(C6*B6),2)</f>
+        <v>5</v>
       </c>
       <c r="T6" s="5">
-        <f>ROUND(N6/(C6*B6),2)</f>
-        <v>4.3300000000000001</v>
-      </c>
-      <c r="U6" s="5">
-        <f>ROUND(H6/(C6*B6),2)</f>
+        <f>ROUND(I6/(C6*B6),2)</f>
         <v>3</v>
       </c>
     </row>
@@ -1786,7 +2097,7 @@
         <v>8</v>
       </c>
       <c r="D7">
-        <v>20.829999999999998</v>
+        <v>20.920000000000002</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1801,7 +2112,7 @@
         <v>0</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="J7">
         <v>6000</v>
@@ -1810,47 +2121,188 @@
         <v>6000</v>
       </c>
       <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>2</v>
+        <v>7000</v>
+      </c>
+      <c r="M7" s="5">
+        <f>IF(H7=1,F7*G7/12,CEILING(ROUND(F7*G7/12/(C7*B7),6),1)*C7*B7)</f>
+        <v>40</v>
       </c>
       <c r="N7" s="5">
-        <f>F7*G7/12</f>
-        <v>34.666666666666664</v>
+        <f>MAX(0,E7+M7-I7)</f>
+        <v>16</v>
       </c>
       <c r="O7" s="5">
-        <f>MAX(0,E7+N7-H7)</f>
-        <v>34.666666666666664</v>
-      </c>
-      <c r="P7" s="5">
-        <f>ROUND((I7+J7+K7+L7)/M7,2)</f>
-        <v>6000</v>
-      </c>
-      <c r="Q7" s="6">
-        <f>P7/(D7*B7)/C7</f>
-        <v>36.005760921747481</v>
+        <f>ROUND(AVERAGE(J7:L7),2)</f>
+        <v>6333.3299999999999</v>
+      </c>
+      <c r="P7" s="6">
+        <f>O7/(D7*B7)/C7</f>
+        <v>37.842554971319309</v>
+      </c>
+      <c r="Q7" s="5">
+        <f>ROUND(N7*P7,2)</f>
+        <v>605.48000000000002</v>
       </c>
       <c r="R7" s="5">
-        <f>ROUND(O7*Q7,2)</f>
-        <v>1248.2</v>
+        <f>ROUND(E7/(C7*B7),2)</f>
+        <v>0</v>
       </c>
       <c r="S7" s="5">
-        <f>ROUND(E7/(C7*B7),2)</f>
-        <v>0</v>
+        <f>ROUND(M7/(C7*B7),2)</f>
+        <v>5</v>
       </c>
       <c r="T7" s="5">
-        <f>ROUND(N7/(C7*B7),2)</f>
-        <v>4.3300000000000001</v>
-      </c>
-      <c r="U7" s="5">
-        <f>ROUND(H7/(C7*B7),2)</f>
+        <f>ROUND(I7/(C7*B7),2)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>8</v>
+      </c>
+      <c r="D8">
+        <v>20.920000000000002</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>208</v>
+      </c>
+      <c r="G8">
+        <v>10</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>6300</v>
+      </c>
+      <c r="L8">
+        <v>6400</v>
+      </c>
+      <c r="M8" s="5">
+        <f>IF(H8=1,F8*G8/12,CEILING(ROUND(F8*G8/12/(C8*B8),6),1)*C8*B8)</f>
+        <v>176</v>
+      </c>
+      <c r="N8" s="5">
+        <f>MAX(0,E8+M8-I8)</f>
+        <v>176</v>
+      </c>
+      <c r="O8" s="5">
+        <f>ROUND(AVERAGE(J8:L8),2)</f>
+        <v>6350</v>
+      </c>
+      <c r="P8" s="6">
+        <f>O8/(D8*B8)/C8</f>
+        <v>37.942160611854682</v>
+      </c>
+      <c r="Q8" s="5">
+        <f>ROUND(N8*P8,2)</f>
+        <v>6677.8199999999997</v>
+      </c>
+      <c r="R8" s="5">
+        <f>ROUND(E8/(C8*B8),2)</f>
+        <v>0</v>
+      </c>
+      <c r="S8" s="5">
+        <f>ROUND(M8/(C8*B8),2)</f>
+        <v>22</v>
+      </c>
+      <c r="T8" s="5">
+        <f>ROUND(I8/(C8*B8),2)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>127</v>
+        <v>52</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>20.920000000000002</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>208</v>
+      </c>
+      <c r="G9">
+        <v>2</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>6000</v>
+      </c>
+      <c r="L9">
+        <v>6000</v>
+      </c>
+      <c r="M9" s="5">
+        <f>IF(H9=1,F9*G9/12,CEILING(ROUND(F9*G9/12/(C9*B9),6),1)*C9*B9)</f>
+        <v>40</v>
+      </c>
+      <c r="N9" s="5">
+        <f>MAX(0,E9+M9-I9)</f>
+        <v>40</v>
+      </c>
+      <c r="O9" s="5">
+        <f>ROUND(AVERAGE(J9:L9),2)</f>
+        <v>6000</v>
+      </c>
+      <c r="P9" s="6">
+        <f>O9/(D9*B9)/C9</f>
+        <v>35.850860420650093</v>
+      </c>
+      <c r="Q9" s="5">
+        <f>ROUND(N9*P9,2)</f>
+        <v>1434.03</v>
+      </c>
+      <c r="R9" s="5">
+        <f>ROUND(E9/(C9*B9),2)</f>
+        <v>0</v>
+      </c>
+      <c r="S9" s="5">
+        <f>ROUND(M9/(C9*B9),2)</f>
+        <v>5</v>
+      </c>
+      <c r="T9" s="5">
+        <f>ROUND(I9/(C9*B9),2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>